<commit_message>
Se hizo el modelo enriquesido de la segunda version del modelo
</commit_message>
<xml_diff>
--- a/Muestreo_de_datos_2.xlsx
+++ b/Muestreo_de_datos_2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0697F228-E35E-498F-9B82-00B1E993C79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0620D41A-B3CE-4D55-BBE2-DF92230490AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="M-CitaServicio" sheetId="16" r:id="rId16"/>
     <sheet name="M-Multa" sheetId="17" r:id="rId17"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1276,7 +1276,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1536,17 +1536,15 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1584,10 +1582,10 @@
     <xf numFmtId="0" fontId="7" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3575,10 +3573,10 @@
       <c r="G2" s="59" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="107" t="s">
+      <c r="H2" s="105" t="s">
         <v>173</v>
       </c>
-      <c r="I2" s="107" t="s">
+      <c r="I2" s="105" t="s">
         <v>174</v>
       </c>
       <c r="J2" s="59" t="s">
@@ -3590,7 +3588,7 @@
       <c r="L2" s="60" t="s">
         <v>177</v>
       </c>
-      <c r="M2" s="108" t="s">
+      <c r="M2" s="106" t="s">
         <v>178</v>
       </c>
     </row>
@@ -3631,7 +3629,7 @@
       <c r="L3" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="M3" s="109" t="s">
+      <c r="M3" s="107" t="s">
         <v>137</v>
       </c>
     </row>
@@ -3654,7 +3652,7 @@
       <c r="G4" s="14">
         <v>3234528921</v>
       </c>
-      <c r="H4" s="106" t="s">
+      <c r="H4" s="104" t="s">
         <v>183</v>
       </c>
       <c r="I4" s="6" t="s">
@@ -3698,7 +3696,7 @@
       <c r="G5" s="14">
         <v>3161657782</v>
       </c>
-      <c r="H5" s="106" t="s">
+      <c r="H5" s="104" t="s">
         <v>187</v>
       </c>
       <c r="I5" s="6" t="s">
@@ -3740,7 +3738,7 @@
       <c r="G6" s="14">
         <v>3119884321</v>
       </c>
-      <c r="H6" s="106" t="s">
+      <c r="H6" s="104" t="s">
         <v>191</v>
       </c>
       <c r="I6" s="6" t="s">
@@ -3780,7 +3778,7 @@
       <c r="G7" s="14">
         <v>4127359182</v>
       </c>
-      <c r="H7" s="106" t="s">
+      <c r="H7" s="104" t="s">
         <v>195</v>
       </c>
       <c r="I7" s="6" t="s">
@@ -3824,7 +3822,7 @@
       <c r="G8" s="14">
         <v>3005544332</v>
       </c>
-      <c r="H8" s="106" t="s">
+      <c r="H8" s="104" t="s">
         <v>201</v>
       </c>
       <c r="I8" s="6" t="s">
@@ -4848,14 +4846,14 @@
     <col min="4" max="4" width="64.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="112" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="110" t="s">
+    <row r="1" spans="1:4" s="110" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="108" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="110" t="s">
+      <c r="B1" s="108" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="111"/>
+      <c r="C1" s="109"/>
     </row>
     <row r="2" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
@@ -4893,7 +4891,7 @@
         <f>'M-HorarioBarbero'!I4</f>
         <v>+57-3245627890-Lunes-09:00-19:00-10:00-16:00</v>
       </c>
-      <c r="C4" s="113">
+      <c r="C4" s="111">
         <v>46265</v>
       </c>
       <c r="D4" s="14" t="str">
@@ -4909,7 +4907,7 @@
         <f>'M-HorarioBarbero'!I5</f>
         <v>+57-3124518923-Martes-09:00-19:00-09:00-15:00</v>
       </c>
-      <c r="C5" s="113">
+      <c r="C5" s="111">
         <v>46091</v>
       </c>
       <c r="D5" s="14" t="str">
@@ -4925,7 +4923,7 @@
         <f>'M-HorarioBarbero'!I6</f>
         <v>+57-3214533321-Jueves-09:00-19:00-13:00-19:00</v>
       </c>
-      <c r="C6" s="113">
+      <c r="C6" s="111">
         <v>46156</v>
       </c>
       <c r="D6" s="14" t="str">
@@ -4941,7 +4939,7 @@
         <f>'M-HorarioBarbero'!I8</f>
         <v>+91-9876543210-Festivo-10:00-15:00-12:00-15:00</v>
       </c>
-      <c r="C7" s="113">
+      <c r="C7" s="111">
         <v>46073</v>
       </c>
       <c r="D7" s="14" t="str">
@@ -4957,7 +4955,7 @@
         <f>'M-HorarioBarbero'!I7</f>
         <v>+91-9876543210-Sábado-08:00-21:00-08:00-14:00</v>
       </c>
-      <c r="C8" s="113">
+      <c r="C8" s="111">
         <v>45983</v>
       </c>
       <c r="D8" s="14" t="str">
@@ -4973,7 +4971,7 @@
         <f>'M-HorarioBarbero'!I6</f>
         <v>+57-3214533321-Jueves-09:00-19:00-13:00-19:00</v>
       </c>
-      <c r="C9" s="113">
+      <c r="C9" s="111">
         <v>46240</v>
       </c>
       <c r="D9" s="14" t="str">
@@ -4989,7 +4987,7 @@
         <f>'M-HorarioBarbero'!I4</f>
         <v>+57-3245627890-Lunes-09:00-19:00-10:00-16:00</v>
       </c>
-      <c r="C10" s="113">
+      <c r="C10" s="111">
         <v>46174</v>
       </c>
       <c r="D10" s="14" t="str">
@@ -5005,7 +5003,7 @@
         <f>'M-HorarioBarbero'!I5</f>
         <v>+57-3124518923-Martes-09:00-19:00-09:00-15:00</v>
       </c>
-      <c r="C11" s="113">
+      <c r="C11" s="111">
         <v>46189</v>
       </c>
       <c r="D11" s="14" t="str">
@@ -5021,7 +5019,7 @@
         <f>'M-HorarioBarbero'!I6</f>
         <v>+57-3214533321-Jueves-09:00-19:00-13:00-19:00</v>
       </c>
-      <c r="C12" s="113">
+      <c r="C12" s="111">
         <v>46205</v>
       </c>
       <c r="D12" s="14" t="str">
@@ -5977,7 +5975,7 @@
       <c r="E2" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F2" s="116" t="s">
+      <c r="F2" s="114" t="s">
         <v>269</v>
       </c>
       <c r="G2" s="10" t="s">
@@ -5988,10 +5986,10 @@
       <c r="A3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="115" t="s">
+      <c r="B3" s="113" t="s">
         <v>271</v>
       </c>
-      <c r="C3" s="115" t="s">
+      <c r="C3" s="113" t="s">
         <v>272</v>
       </c>
       <c r="D3" s="85" t="s">
@@ -6007,15 +6005,15 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="14">
         <v>1</v>
       </c>
-      <c r="B4" s="114" t="str">
+      <c r="B4" s="112" t="str">
         <f>'M-Cita'!P4</f>
         <v>+57-3245627890-Lunes-09:00-19:00-10:00-16:00-31/08/2026-10:00</v>
       </c>
-      <c r="C4" s="114" t="str">
+      <c r="C4" s="112" t="str">
         <f>'M-BarberoServicio'!G4</f>
         <v>Juan García-Motilada</v>
       </c>
@@ -6036,7 +6034,7 @@
         <v>+57-3245627890-Lunes-09:00-19:00-10:00-16:00-31/08/2026-10:00-Juan García-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>2</v>
       </c>
@@ -6181,7 +6179,7 @@
         <v>+91-9876543210-Festivo-10:00-15:00-12:00-15:00-20/02/2026-14:00-Andres Ramirez-Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>7</v>
       </c>
@@ -6210,7 +6208,7 @@
         <v>+57-3245627890-Lunes-09:00-19:00-10:00-16:00-01/06/2026-10:00-Juan García-Motilada</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>8</v>
       </c>
@@ -6531,8 +6529,8 @@
         <f>'M-Cita'!H6</f>
         <v>0.55208333333333304</v>
       </c>
-      <c r="F4" s="119">
-        <v>46233</v>
+      <c r="F4" s="118">
+        <v>46233.416666666664</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>83</v>
@@ -6667,7 +6665,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="F10" s="120"/>
+      <c r="F10" s="117"/>
     </row>
     <row r="14" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="95"/>
@@ -6694,13 +6692,13 @@
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="117"/>
+      <c r="A18" s="115"/>
       <c r="B18" s="18" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="118"/>
+      <c r="A19" s="116"/>
       <c r="B19" s="18" t="s">
         <v>294</v>
       </c>
@@ -6778,14 +6776,14 @@
       <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
     </row>
     <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="102" t="s">
+      <c r="B3" s="101" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="4">
@@ -6794,14 +6792,12 @@
       <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="105"/>
-      <c r="F3" s="105"/>
     </row>
     <row r="4" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="101" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="103" t="s">
+      <c r="B4" s="102" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="6">
@@ -6810,14 +6806,12 @@
       <c r="D4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
     </row>
     <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="101" t="s">
+      <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="103" t="s">
+      <c r="B5" s="102" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="6">
@@ -6826,14 +6820,12 @@
       <c r="D5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="105"/>
-      <c r="F5" s="105"/>
     </row>
     <row r="6" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="101" t="s">
+      <c r="A6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="103" t="s">
+      <c r="B6" s="102" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="6">
@@ -6842,14 +6834,12 @@
       <c r="D6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="105"/>
-      <c r="F6" s="105"/>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="101" t="s">
+      <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="103" t="s">
+      <c r="B7" s="102" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="6">
@@ -6858,14 +6848,12 @@
       <c r="D7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="105"/>
-      <c r="F7" s="105"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="101" t="s">
+      <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="103" t="s">
+      <c r="B8" s="102" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="6">
@@ -6874,14 +6862,12 @@
       <c r="D8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="105"/>
-      <c r="F8" s="105"/>
     </row>
     <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="101" t="s">
+      <c r="A9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="103" t="s">
+      <c r="B9" s="102" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="6">
@@ -6890,14 +6876,12 @@
       <c r="D9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="105"/>
-      <c r="F9" s="105"/>
     </row>
     <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="101" t="s">
+      <c r="A10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="103" t="s">
+      <c r="B10" s="102" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="6">
@@ -6906,14 +6890,12 @@
       <c r="D10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="105"/>
-      <c r="F10" s="105"/>
     </row>
     <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="101" t="s">
+      <c r="A11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="103" t="s">
+      <c r="B11" s="102" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="6">
@@ -6922,14 +6904,12 @@
       <c r="D11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="105"/>
-      <c r="F11" s="105"/>
     </row>
     <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="101" t="s">
+      <c r="A12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="103" t="s">
+      <c r="B12" s="102" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="6">
@@ -6938,14 +6918,12 @@
       <c r="D12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="105"/>
-      <c r="F12" s="105"/>
     </row>
     <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="101" t="s">
+      <c r="A13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="103" t="s">
+      <c r="B13" s="102" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="6">
@@ -6954,14 +6932,12 @@
       <c r="D13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E13" s="105"/>
-      <c r="F13" s="105"/>
     </row>
     <row r="14" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="101" t="s">
+      <c r="A14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="103" t="s">
+      <c r="B14" s="102" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="6">
@@ -6970,14 +6946,12 @@
       <c r="D14" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
     </row>
     <row r="15" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="101" t="s">
+      <c r="A15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="103" t="s">
+      <c r="B15" s="102" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="6">
@@ -6986,14 +6960,12 @@
       <c r="D15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="105"/>
-      <c r="F15" s="105"/>
     </row>
     <row r="16" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="101" t="s">
+      <c r="A16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="103" t="s">
+      <c r="B16" s="102" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="6">
@@ -7002,14 +6974,12 @@
       <c r="D16" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="105"/>
-      <c r="F16" s="105"/>
-    </row>
-    <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="101" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="103" t="s">
+      <c r="B17" s="102" t="s">
         <v>36</v>
       </c>
       <c r="C17" s="6">
@@ -7018,8 +6988,6 @@
       <c r="D17" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="105"/>
-      <c r="F17" s="105"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>